<commit_message>
Added .gitignore and made changes
</commit_message>
<xml_diff>
--- a/Business/Data.xlsx
+++ b/Business/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1a98318606382685/Desktop/My Automations/ID Card Automation/Business/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{25BFEC68-8685-4EEC-8223-8F1A164D547E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62F5CECF-EABE-4C2E-9E7C-38F93A0DBC32}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{25BFEC68-8685-4EEC-8223-8F1A164D547E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36DA9CE2-B4E4-4A8E-B51E-5BE5CB06134D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{991AF25C-59D6-4B86-8DBE-D954CDD9AFD9}"/>
+    <workbookView xWindow="5556" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{991AF25C-59D6-4B86-8DBE-D954CDD9AFD9}"/>
   </bookViews>
   <sheets>
     <sheet name="CardData" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
   <si>
     <t>No</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>Sheila Dever</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -177,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -200,11 +203,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -219,6 +233,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -236,6 +253,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -535,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7414E961-F0F5-4A4D-BA98-8F48FCDB5978}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" customWidth="1"/>
@@ -544,10 +565,10 @@
     <col min="4" max="4" width="16.109375" customWidth="1"/>
     <col min="5" max="5" width="17.44140625" customWidth="1"/>
     <col min="6" max="6" width="19.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" customWidth="1"/>
+    <col min="7" max="7" width="99.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -566,8 +587,11 @@
       <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G1" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -587,7 +611,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -607,7 +631,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -627,7 +651,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -647,7 +671,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -667,7 +691,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -687,7 +711,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -705,7 +729,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -725,7 +749,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -745,7 +769,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -765,7 +789,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -785,7 +809,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -805,7 +829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -823,7 +847,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -841,7 +865,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>

</xml_diff>